<commit_message>
Add quote summary functionality and refactor related steps Added method for selecting radio buttons in base page Added locator.press("Tab") in method type_text to simulate real user behavior Changed some of the fill methods with custom type_text method
</commit_message>
<xml_diff>
--- a/testdata/static/AutoData.xlsx
+++ b/testdata/static/AutoData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MasterTest\Sandbox-master\src\test_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projekti\SandboxPlaywright\testdata\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9340690-2668-46A9-B772-7CAA4EA1DF0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C4CE6B3-35D9-4D61-BC54-E0C61FE8F48E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24315" yWindow="3600" windowWidth="19200" windowHeight="11175" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21285" yWindow="3720" windowWidth="19200" windowHeight="11175" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Policy_DataDStatus" sheetId="13" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="196">
   <si>
     <t>Common Data for Quotes, Customer, PolicyInformation, LocationCoverage and Rate pages</t>
   </si>
@@ -628,6 +628,9 @@
   </si>
   <si>
     <t>2017</t>
+  </si>
+  <si>
+    <t>BillingMethod</t>
   </si>
 </sst>
 </file>
@@ -635,7 +638,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -781,17 +784,17 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1087,21 +1090,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
@@ -1724,21 +1727,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
@@ -2350,7 +2353,7 @@
   <dimension ref="A1:AJ12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="9" max="9" width="8.7265625" style="26"/>
+    <col min="9" max="9" width="8.7265625" style="24"/>
     <col min="14" max="14" width="24.453125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2365,7 +2368,7 @@
       <c r="F1" s="21"/>
       <c r="G1" s="21"/>
       <c r="H1" s="21"/>
-      <c r="I1" s="24"/>
+      <c r="I1" s="22"/>
       <c r="J1" s="21"/>
       <c r="K1" s="21"/>
       <c r="L1" s="21"/>
@@ -2419,7 +2422,7 @@
       <c r="H2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="25" t="s">
+      <c r="I2" s="23" t="s">
         <v>10</v>
       </c>
       <c r="J2" s="2" t="s">
@@ -2435,7 +2438,7 @@
         <v>14</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>15</v>
+        <v>195</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>16</v>
@@ -3626,21 +3629,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="25" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
@@ -3803,21 +3806,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="25" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
@@ -3976,27 +3979,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:37" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
-      <c r="S1" s="23"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
+      <c r="O1" s="26"/>
+      <c r="P1" s="26"/>
+      <c r="Q1" s="26"/>
+      <c r="R1" s="26"/>
+      <c r="S1" s="26"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
       <c r="V1" s="1"/>
@@ -4914,22 +4917,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>

</xml_diff>